<commit_message>
27/05: Actualización gráficos de resultados con bandas de confianza por simulacion de monte carlo
</commit_message>
<xml_diff>
--- a/Códigos_modelo_Coleman/optimizacion_pymoo/resultados_buenos/Resultados estimaciones utilizados.xlsx
+++ b/Códigos_modelo_Coleman/optimizacion_pymoo/resultados_buenos/Resultados estimaciones utilizados.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\p-mfolch\Documents\Proyecto_Tintos_CyT\Códigos_oficiales_model2\optimizacion_pymoo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\p-mfolch\Documents\Proyecto_Tintos_CyT\Códigos_modelo_Coleman\optimizacion_pymoo\resultados_buenos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43B45062-1951-4246-ACA8-6F8EEC7BC287}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82297BB4-C89D-48E3-BF65-2FFA438885BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,35 +20,40 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$Y$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Hoja1 (3)'!$A$1:$Y$1</definedName>
     <definedName name="_xlchart.v1.0" hidden="1">Hoja1!$V$2:$V$21</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">Hoja1!$Y$1</definedName>
-    <definedName name="_xlchart.v1.10" hidden="1">Hoja1!$Y$2:$Y$21</definedName>
-    <definedName name="_xlchart.v1.11" hidden="1">Hoja1!$X$1</definedName>
-    <definedName name="_xlchart.v1.12" hidden="1">Hoja1!$X$2:$X$21</definedName>
-    <definedName name="_xlchart.v1.13" hidden="1">Hoja1!$W$1</definedName>
-    <definedName name="_xlchart.v1.14" hidden="1">Hoja1!$W$2:$W$21</definedName>
-    <definedName name="_xlchart.v1.15" hidden="1">'Hoja1 (3)'!$W$1</definedName>
-    <definedName name="_xlchart.v1.16" hidden="1">'Hoja1 (3)'!$W$2:$W$21</definedName>
-    <definedName name="_xlchart.v1.17" hidden="1">'Hoja1 (3)'!$W$1</definedName>
-    <definedName name="_xlchart.v1.18" hidden="1">'Hoja1 (3)'!$W$2:$W$21</definedName>
-    <definedName name="_xlchart.v1.19" hidden="1">'Hoja1 (3)'!$X$1</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">Hoja1!$Y$2:$Y$21</definedName>
-    <definedName name="_xlchart.v1.20" hidden="1">'Hoja1 (3)'!$X$2:$X$21</definedName>
-    <definedName name="_xlchart.v1.21" hidden="1">'Hoja1 (3)'!$Y$1</definedName>
-    <definedName name="_xlchart.v1.22" hidden="1">'Hoja1 (3)'!$Y$2:$Y$21</definedName>
-    <definedName name="_xlchart.v1.23" hidden="1">'Hoja1 (3)'!$V$2:$V$21</definedName>
-    <definedName name="_xlchart.v1.24" hidden="1">'Hoja1 (3)'!$V$1</definedName>
-    <definedName name="_xlchart.v1.25" hidden="1">'Hoja1 (3)'!$V$2:$V$21</definedName>
-    <definedName name="_xlchart.v1.26" hidden="1">'Hoja1 (3)'!$Y$1</definedName>
-    <definedName name="_xlchart.v1.27" hidden="1">'Hoja1 (3)'!$Y$2:$Y$21</definedName>
-    <definedName name="_xlchart.v1.28" hidden="1">'Hoja1 (3)'!$X$1</definedName>
-    <definedName name="_xlchart.v1.29" hidden="1">'Hoja1 (3)'!$X$2:$X$21</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">Hoja1!$V$1</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">Hoja1!$V$2:$V$21</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">Hoja1!$X$1</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">Hoja1!$X$2:$X$21</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">Hoja1!$W$1</definedName>
-    <definedName name="_xlchart.v1.8" hidden="1">Hoja1!$W$2:$W$21</definedName>
-    <definedName name="_xlchart.v1.9" hidden="1">Hoja1!$Y$1</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Hoja1!$V$2:$V$21</definedName>
+    <definedName name="_xlchart.v1.10" hidden="1">Hoja1!$X$1</definedName>
+    <definedName name="_xlchart.v1.11" hidden="1">Hoja1!$X$2:$X$21</definedName>
+    <definedName name="_xlchart.v1.12" hidden="1">Hoja1!$V$2:$V$21</definedName>
+    <definedName name="_xlchart.v1.13" hidden="1">Hoja1!$V$1</definedName>
+    <definedName name="_xlchart.v1.14" hidden="1">Hoja1!$V$2:$V$21</definedName>
+    <definedName name="_xlchart.v1.15" hidden="1">Hoja1!$X$1</definedName>
+    <definedName name="_xlchart.v1.16" hidden="1">Hoja1!$X$2:$X$21</definedName>
+    <definedName name="_xlchart.v1.17" hidden="1">Hoja1!$Y$1</definedName>
+    <definedName name="_xlchart.v1.18" hidden="1">Hoja1!$Y$2:$Y$21</definedName>
+    <definedName name="_xlchart.v1.19" hidden="1">Hoja1!$V$2:$V$21</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Hoja1!$Y$1</definedName>
+    <definedName name="_xlchart.v1.20" hidden="1">'Hoja1 (3)'!$V$1</definedName>
+    <definedName name="_xlchart.v1.21" hidden="1">'Hoja1 (3)'!$V$2:$V$21</definedName>
+    <definedName name="_xlchart.v1.22" hidden="1">'Hoja1 (3)'!$V$2:$V$21</definedName>
+    <definedName name="_xlchart.v1.23" hidden="1">'Hoja1 (3)'!$W$1</definedName>
+    <definedName name="_xlchart.v1.24" hidden="1">'Hoja1 (3)'!$W$2:$W$21</definedName>
+    <definedName name="_xlchart.v1.25" hidden="1">'Hoja1 (3)'!$X$1</definedName>
+    <definedName name="_xlchart.v1.26" hidden="1">'Hoja1 (3)'!$X$2:$X$21</definedName>
+    <definedName name="_xlchart.v1.27" hidden="1">'Hoja1 (3)'!$X$1</definedName>
+    <definedName name="_xlchart.v1.28" hidden="1">'Hoja1 (3)'!$X$2:$X$21</definedName>
+    <definedName name="_xlchart.v1.29" hidden="1">'Hoja1 (3)'!$Y$1</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">Hoja1!$Y$2:$Y$21</definedName>
+    <definedName name="_xlchart.v1.30" hidden="1">'Hoja1 (3)'!$Y$2:$Y$21</definedName>
+    <definedName name="_xlchart.v1.31" hidden="1">'Hoja1 (3)'!$W$1</definedName>
+    <definedName name="_xlchart.v1.32" hidden="1">'Hoja1 (3)'!$W$2:$W$21</definedName>
+    <definedName name="_xlchart.v1.33" hidden="1">'Hoja1 (3)'!$Y$1</definedName>
+    <definedName name="_xlchart.v1.34" hidden="1">'Hoja1 (3)'!$Y$2:$Y$21</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">Hoja1!$W$1</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">Hoja1!$W$2:$W$21</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">Hoja1!$Y$1</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">Hoja1!$Y$2:$Y$21</definedName>
+    <definedName name="_xlchart.v1.8" hidden="1">Hoja1!$W$1</definedName>
+    <definedName name="_xlchart.v1.9" hidden="1">Hoja1!$W$2:$W$21</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -338,9 +343,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.00000000"/>
     <numFmt numFmtId="165" formatCode="0.000000000"/>
+    <numFmt numFmtId="168" formatCode="0.0000"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -451,7 +457,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -463,6 +469,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -526,7 +533,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.0</cx:f>
+        <cx:f>_xlchart.v1.12</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -562,6 +569,21 @@
     <cx:plotArea>
       <cx:plotAreaRegion>
         <cx:series layoutId="boxWhisker" uniqueId="{C6BD7690-477A-45D1-867D-425763C21062}">
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Kn 20 datos</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:ln>
+          </cx:spPr>
           <cx:dataId val="0"/>
           <cx:layoutPr>
             <cx:visibility meanLine="0" meanMarker="1" nonoutliers="0" outliers="1"/>
@@ -579,6 +601,7 @@
         <cx:tickLabels/>
       </cx:axis>
     </cx:plotArea>
+    <cx:legend pos="b" align="ctr" overlay="0"/>
   </cx:chart>
 </cx:chartSpace>
 </file>
@@ -588,7 +611,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.25</cx:f>
+        <cx:f>_xlchart.v1.21</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -598,7 +621,7 @@
         <cx:series layoutId="clusteredColumn" uniqueId="{00000001-BC7E-4971-A06E-D207053F9DAB}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.24</cx:f>
+              <cx:f>_xlchart.v1.20</cx:f>
               <cx:v>Kn</cx:v>
             </cx:txData>
           </cx:tx>
@@ -627,7 +650,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.16</cx:f>
+        <cx:f>_xlchart.v1.32</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -665,7 +688,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{0F116D08-654B-4473-A6FE-BF660B39F4C3}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.15</cx:f>
+              <cx:f>_xlchart.v1.31</cx:f>
               <cx:v>Yxn</cx:v>
             </cx:txData>
           </cx:tx>
@@ -694,7 +717,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.18</cx:f>
+        <cx:f>_xlchart.v1.24</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -704,7 +727,7 @@
         <cx:series layoutId="clusteredColumn" uniqueId="{E326187D-54D7-4466-ACB4-35ABCDAD8652}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.17</cx:f>
+              <cx:f>_xlchart.v1.23</cx:f>
               <cx:v>Yxn</cx:v>
             </cx:txData>
           </cx:tx>
@@ -733,7 +756,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.20</cx:f>
+        <cx:f>_xlchart.v1.26</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -771,7 +794,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{81576D69-9D5A-4D7E-BAF0-D74822440E08}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.19</cx:f>
+              <cx:f>_xlchart.v1.25</cx:f>
               <cx:v>Yes</cx:v>
             </cx:txData>
           </cx:tx>
@@ -800,7 +823,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.29</cx:f>
+        <cx:f>_xlchart.v1.28</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -810,7 +833,7 @@
         <cx:series layoutId="clusteredColumn" uniqueId="{B7A9DC36-E507-4C9C-9C7A-E7D5B042F55A}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.28</cx:f>
+              <cx:f>_xlchart.v1.27</cx:f>
               <cx:v>Yes</cx:v>
             </cx:txData>
           </cx:tx>
@@ -839,7 +862,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.27</cx:f>
+        <cx:f>_xlchart.v1.34</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -877,7 +900,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{45E274BE-57DD-456B-BB92-E707190C011F}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.26</cx:f>
+              <cx:f>_xlchart.v1.33</cx:f>
               <cx:v>Ks</cx:v>
             </cx:txData>
           </cx:tx>
@@ -906,7 +929,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.22</cx:f>
+        <cx:f>_xlchart.v1.30</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -916,7 +939,7 @@
         <cx:series layoutId="clusteredColumn" uniqueId="{6A3144A3-5D7D-4603-8BC6-AB23FF9069ED}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.21</cx:f>
+              <cx:f>_xlchart.v1.29</cx:f>
               <cx:v>Ks</cx:v>
             </cx:txData>
           </cx:tx>
@@ -945,7 +968,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.4</cx:f>
+        <cx:f>_xlchart.v1.14</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -955,7 +978,7 @@
         <cx:series layoutId="clusteredColumn" uniqueId="{00000001-BC7E-4971-A06E-D207053F9DAB}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.3</cx:f>
+              <cx:f>_xlchart.v1.13</cx:f>
               <cx:v>Kn</cx:v>
             </cx:txData>
           </cx:tx>
@@ -984,7 +1007,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.14</cx:f>
+        <cx:f>_xlchart.v1.5</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -1022,10 +1045,19 @@
         <cx:series layoutId="boxWhisker" uniqueId="{0F116D08-654B-4473-A6FE-BF660B39F4C3}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.13</cx:f>
-              <cx:v>Yxn</cx:v>
+              <cx:v>Yxn 20 datos</cx:v>
             </cx:txData>
           </cx:tx>
+          <cx:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:ln>
+          </cx:spPr>
           <cx:dataId val="0"/>
           <cx:layoutPr>
             <cx:statistics quartileMethod="exclusive"/>
@@ -1042,6 +1074,7 @@
         <cx:tickLabels/>
       </cx:axis>
     </cx:plotArea>
+    <cx:legend pos="b" align="ctr" overlay="0"/>
   </cx:chart>
 </cx:chartSpace>
 </file>
@@ -1051,7 +1084,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.8</cx:f>
+        <cx:f>_xlchart.v1.9</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -1061,7 +1094,7 @@
         <cx:series layoutId="clusteredColumn" uniqueId="{E326187D-54D7-4466-ACB4-35ABCDAD8652}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.7</cx:f>
+              <cx:f>_xlchart.v1.8</cx:f>
               <cx:v>Yxn</cx:v>
             </cx:txData>
           </cx:tx>
@@ -1090,7 +1123,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.12</cx:f>
+        <cx:f>_xlchart.v1.11</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -1128,10 +1161,19 @@
         <cx:series layoutId="boxWhisker" uniqueId="{81576D69-9D5A-4D7E-BAF0-D74822440E08}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.11</cx:f>
-              <cx:v>Yes</cx:v>
+              <cx:v>Yes 20 datos</cx:v>
             </cx:txData>
           </cx:tx>
+          <cx:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent3"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:ln>
+          </cx:spPr>
           <cx:dataId val="0"/>
           <cx:layoutPr>
             <cx:statistics quartileMethod="exclusive"/>
@@ -1148,6 +1190,7 @@
         <cx:tickLabels/>
       </cx:axis>
     </cx:plotArea>
+    <cx:legend pos="b" align="ctr" overlay="0"/>
   </cx:chart>
 </cx:chartSpace>
 </file>
@@ -1157,7 +1200,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.6</cx:f>
+        <cx:f>_xlchart.v1.16</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -1167,7 +1210,7 @@
         <cx:series layoutId="clusteredColumn" uniqueId="{B7A9DC36-E507-4C9C-9C7A-E7D5B042F55A}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.5</cx:f>
+              <cx:f>_xlchart.v1.15</cx:f>
               <cx:v>Yes</cx:v>
             </cx:txData>
           </cx:tx>
@@ -1196,7 +1239,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.10</cx:f>
+        <cx:f>_xlchart.v1.7</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -1234,10 +1277,19 @@
         <cx:series layoutId="boxWhisker" uniqueId="{45E274BE-57DD-456B-BB92-E707190C011F}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.9</cx:f>
-              <cx:v>Ks</cx:v>
+              <cx:v>Ks 20 datos</cx:v>
             </cx:txData>
           </cx:tx>
+          <cx:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent4"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:ln>
+          </cx:spPr>
           <cx:dataId val="0"/>
           <cx:layoutPr>
             <cx:statistics quartileMethod="exclusive"/>
@@ -1249,11 +1301,12 @@
         <cx:tickLabels/>
       </cx:axis>
       <cx:axis id="1">
-        <cx:valScaling/>
+        <cx:valScaling max="100"/>
         <cx:majorGridlines/>
         <cx:tickLabels/>
       </cx:axis>
     </cx:plotArea>
+    <cx:legend pos="b" align="ctr" overlay="0"/>
   </cx:chart>
 </cx:chartSpace>
 </file>
@@ -1263,7 +1316,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.2</cx:f>
+        <cx:f>_xlchart.v1.3</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -1273,7 +1326,7 @@
         <cx:series layoutId="clusteredColumn" uniqueId="{6A3144A3-5D7D-4603-8BC6-AB23FF9069ED}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.1</cx:f>
+              <cx:f>_xlchart.v1.2</cx:f>
               <cx:v>Ks</cx:v>
             </cx:txData>
           </cx:tx>
@@ -1302,7 +1355,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.23</cx:f>
+        <cx:f>_xlchart.v1.22</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -10190,13 +10243,13 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>411480</xdr:colOff>
       <xdr:row>25</xdr:row>
-      <xdr:rowOff>171450</xdr:rowOff>
+      <xdr:rowOff>44450</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>228600</xdr:colOff>
+      <xdr:colOff>133080</xdr:colOff>
       <xdr:row>40</xdr:row>
-      <xdr:rowOff>171450</xdr:rowOff>
+      <xdr:rowOff>130450</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
@@ -10232,8 +10285,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="11597640" y="4781550"/>
-              <a:ext cx="2255520" cy="2743200"/>
+              <a:off x="11595947" y="4743450"/>
+              <a:ext cx="2160000" cy="2880000"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -10344,15 +10397,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>502920</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>22860</xdr:rowOff>
+      <xdr:colOff>257386</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>56727</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
-      <xdr:colOff>320040</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>22860</xdr:rowOff>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>588586</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>142727</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
@@ -10388,8 +10441,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="14127480" y="4815840"/>
-              <a:ext cx="2255520" cy="2743200"/>
+              <a:off x="13880253" y="4755727"/>
+              <a:ext cx="2160000" cy="2880000"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -10500,15 +10553,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>25</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>30480</xdr:rowOff>
+      <xdr:colOff>135467</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>47414</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>198120</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>30480</xdr:rowOff>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>466667</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>133414</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
@@ -10544,8 +10597,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="16443960" y="4823460"/>
-              <a:ext cx="2255520" cy="2743200"/>
+              <a:off x="16196734" y="4746414"/>
+              <a:ext cx="2160000" cy="2880000"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -10655,16 +10708,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>411480</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>15240</xdr:rowOff>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>563880</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>40641</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>33</xdr:col>
-      <xdr:colOff>228600</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>15240</xdr:rowOff>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>285480</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>126641</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
@@ -10700,8 +10753,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="18912840" y="4808220"/>
-              <a:ext cx="2255520" cy="2743200"/>
+              <a:off x="18453947" y="4739641"/>
+              <a:ext cx="2160000" cy="2880000"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -11709,6 +11762,10 @@
   <cols>
     <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="10.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -13243,37 +13300,37 @@
       </c>
     </row>
     <row r="24" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="V24">
+      <c r="V24" s="11">
         <f>MEDIAN(V2:V21)</f>
         <v>7.3482996934971247E-4</v>
       </c>
-      <c r="W24">
+      <c r="W24" s="11">
         <f t="shared" ref="W24:Y24" si="1">MEDIAN(W2:W21)</f>
         <v>20.310448257131583</v>
       </c>
-      <c r="X24">
+      <c r="X24" s="11">
         <f t="shared" si="1"/>
         <v>0.3715872236384351</v>
       </c>
-      <c r="Y24">
+      <c r="Y24" s="11">
         <f t="shared" si="1"/>
         <v>17.268174566317164</v>
       </c>
     </row>
     <row r="25" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="V25">
+      <c r="V25" s="11">
         <f>STDEVA(V2:V21)</f>
         <v>6.3777506162885321E-4</v>
       </c>
-      <c r="W25">
+      <c r="W25" s="11">
         <f t="shared" ref="W25:Y25" si="2">STDEVA(W2:W21)</f>
         <v>8.5631716627075409</v>
       </c>
-      <c r="X25">
+      <c r="X25" s="11">
         <f t="shared" si="2"/>
         <v>3.9531802927071397E-2</v>
       </c>
-      <c r="Y25">
+      <c r="Y25" s="11">
         <f t="shared" si="2"/>
         <v>30.113328264384752</v>
       </c>

</xml_diff>